<commit_message>
Atualizando regras n telco especificas
</commit_message>
<xml_diff>
--- a/data/Tabela_cClass.xlsx
+++ b/data/Tabela_cClass.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875407B2-424D-40CB-AB89-4FD043D43A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B87D307D-3937-4D8F-B178-1D4F3D007F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Telco" sheetId="3" r:id="rId1"/>
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Não Tributado'!$A$1:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Telco!$A$1:$E$36</definedName>
   </definedNames>
-  <calcPr calcId="191029" refMode="R1C1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="135">
   <si>
     <t>Grupo/Código</t>
   </si>
@@ -190,9 +190,6 @@
     <t>0450101</t>
   </si>
   <si>
-    <t>Serviços Combinados (dados, voz, mensagens e outros)</t>
-  </si>
-  <si>
     <t>0500101</t>
   </si>
   <si>
@@ -428,6 +425,21 @@
   </si>
   <si>
     <t>NAO TRIBUTADO</t>
+  </si>
+  <si>
+    <t>000</t>
+  </si>
+  <si>
+    <t>000001</t>
+  </si>
+  <si>
+    <t>Serviços Combinados (dados</t>
+  </si>
+  <si>
+    <t>410</t>
+  </si>
+  <si>
+    <t>410999</t>
   </si>
 </sst>
 </file>
@@ -438,7 +450,7 @@
     <numFmt numFmtId="164" formatCode="000"/>
     <numFmt numFmtId="165" formatCode="000000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -460,19 +472,13 @@
     <font>
       <u/>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -482,12 +488,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -504,7 +504,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -512,12 +512,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -862,9 +857,9 @@
   <cols>
     <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="55.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" style="3" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -876,16 +871,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>123</v>
-      </c>
       <c r="F1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -895,17 +890,17 @@
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="7">
-        <v>0</v>
-      </c>
-      <c r="E2" s="8">
-        <v>2</v>
+      <c r="C2" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -915,17 +910,17 @@
       <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D3" s="7">
-        <v>0</v>
-      </c>
-      <c r="E3" s="12">
-        <v>1</v>
+      <c r="C3" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -935,17 +930,17 @@
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D4" s="7">
-        <v>0</v>
-      </c>
-      <c r="E4" s="8">
-        <v>1</v>
+      <c r="C4" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -955,17 +950,17 @@
       <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D5" s="7">
-        <v>0</v>
-      </c>
-      <c r="E5" s="8">
-        <v>1</v>
+      <c r="C5" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -975,17 +970,17 @@
       <c r="B6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D6" s="7">
-        <v>0</v>
-      </c>
-      <c r="E6" s="8">
-        <v>1</v>
+      <c r="C6" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -995,17 +990,17 @@
       <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D7" s="7">
-        <v>0</v>
-      </c>
-      <c r="E7" s="8">
-        <v>1</v>
+      <c r="C7" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1015,17 +1010,17 @@
       <c r="B8" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D8" s="7">
-        <v>0</v>
-      </c>
-      <c r="E8" s="8">
-        <v>1</v>
+      <c r="C8" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1036,16 +1031,16 @@
         <v>17</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D9" s="7">
-        <v>0</v>
-      </c>
-      <c r="E9" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1056,16 +1051,16 @@
         <v>19</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D10" s="7">
-        <v>0</v>
-      </c>
-      <c r="E10" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1076,16 +1071,16 @@
         <v>21</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D11" s="7">
-        <v>0</v>
-      </c>
-      <c r="E11" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1095,17 +1090,17 @@
       <c r="B12" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D12" s="7">
-        <v>0</v>
-      </c>
-      <c r="E12" s="8">
-        <v>1</v>
+      <c r="C12" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1115,17 +1110,17 @@
       <c r="B13" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D13" s="7">
-        <v>0</v>
-      </c>
-      <c r="E13" s="8">
-        <v>1</v>
+      <c r="C13" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1135,17 +1130,17 @@
       <c r="B14" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D14" s="7">
-        <v>0</v>
-      </c>
-      <c r="E14" s="8">
-        <v>1</v>
+      <c r="C14" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1155,17 +1150,17 @@
       <c r="B15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D15" s="7">
-        <v>0</v>
-      </c>
-      <c r="E15" s="8">
-        <v>1</v>
+      <c r="C15" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1175,17 +1170,17 @@
       <c r="B16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D16" s="7">
-        <v>0</v>
-      </c>
-      <c r="E16" s="8">
-        <v>1</v>
+      <c r="C16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1195,17 +1190,17 @@
       <c r="B17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D17" s="7">
-        <v>0</v>
-      </c>
-      <c r="E17" s="8">
-        <v>1</v>
+      <c r="C17" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1215,17 +1210,17 @@
       <c r="B18" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D18" s="7">
-        <v>0</v>
-      </c>
-      <c r="E18" s="8">
-        <v>1</v>
+      <c r="C18" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1236,16 +1231,16 @@
         <v>37</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D19" s="7">
-        <v>0</v>
-      </c>
-      <c r="E19" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="5" customFormat="1" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -1256,16 +1251,16 @@
         <v>39</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D20" s="7">
-        <v>0</v>
-      </c>
-      <c r="E20" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1276,16 +1271,16 @@
         <v>41</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D21" s="7">
-        <v>0</v>
-      </c>
-      <c r="E21" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1295,17 +1290,17 @@
       <c r="B22" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D22" s="7">
-        <v>0</v>
-      </c>
-      <c r="E22" s="8">
-        <v>1</v>
+      <c r="C22" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1315,17 +1310,17 @@
       <c r="B23" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D23" s="7">
-        <v>0</v>
-      </c>
-      <c r="E23" s="8">
-        <v>1</v>
+      <c r="C23" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1335,17 +1330,17 @@
       <c r="B24" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D24" s="7">
-        <v>0</v>
-      </c>
-      <c r="E24" s="8">
-        <v>1</v>
+      <c r="C24" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
@@ -1355,672 +1350,672 @@
       <c r="B25" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D25" s="7">
-        <v>0</v>
-      </c>
-      <c r="E25" s="8">
-        <v>1</v>
+      <c r="C25" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="4" t="s">
         <v>50</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>51</v>
+        <v>132</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D26" s="7">
-        <v>123</v>
-      </c>
-      <c r="E26" s="8">
-        <v>123456</v>
+        <v>123</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D27" s="7">
-        <v>0</v>
-      </c>
-      <c r="E27" s="8">
-        <v>1</v>
+      <c r="C27" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D28" s="7">
-        <v>0</v>
-      </c>
-      <c r="E28" s="8">
-        <v>1</v>
+      <c r="C28" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="29" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>57</v>
-      </c>
       <c r="C29" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D29" s="7">
-        <v>0</v>
-      </c>
-      <c r="E29" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B30" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="4" t="s">
-        <v>59</v>
-      </c>
       <c r="C30" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D30" s="7">
-        <v>0</v>
-      </c>
-      <c r="E30" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="31" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="4" t="s">
-        <v>61</v>
-      </c>
       <c r="C31" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D31" s="7">
-        <v>0</v>
-      </c>
-      <c r="E31" s="8">
-        <v>1</v>
+        <v>123</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D32" s="7">
-        <v>0</v>
-      </c>
-      <c r="E32" s="8">
-        <v>1</v>
+      <c r="C32" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D33" s="7">
-        <v>0</v>
-      </c>
-      <c r="E33" s="8">
-        <v>1</v>
+      <c r="C33" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D34" s="7">
-        <v>0</v>
-      </c>
-      <c r="E34" s="8">
-        <v>1</v>
+      <c r="C34" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D35" s="7">
-        <v>0</v>
-      </c>
-      <c r="E35" s="8">
-        <v>1</v>
+      <c r="C35" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="36" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="D36" s="7">
-        <v>0</v>
-      </c>
-      <c r="E36" s="8">
-        <v>1</v>
+      <c r="C36" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>131</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="G36" s="11"/>
+        <v>127</v>
+      </c>
+      <c r="G36" s="7"/>
     </row>
     <row r="37" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="C37" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="38" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="C38" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="39" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B39" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="C39" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="40" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>73</v>
-      </c>
       <c r="C40" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="C41" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B42" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="C42" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="43" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B43" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="C43" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>89</v>
-      </c>
       <c r="C44" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B45" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>91</v>
-      </c>
       <c r="C45" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>93</v>
-      </c>
       <c r="C46" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="47" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B47" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="C47" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="F47" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F48" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E49" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F49" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="C47" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="F47" s="5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="B48" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="C48" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D48" s="11">
-        <v>410</v>
-      </c>
-      <c r="E48" s="11">
-        <v>410999</v>
-      </c>
-      <c r="F48" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="C49" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D49" s="11">
-        <v>410</v>
-      </c>
-      <c r="E49" s="11">
-        <v>410999</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="10" t="s">
+      <c r="B50" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B50" s="10" t="s">
+      <c r="C50" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E50" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F50" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="C50" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D50" s="5">
-        <v>410</v>
-      </c>
-      <c r="E50" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F50" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="10" t="s">
+      <c r="B51" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B51" s="10" t="s">
+      <c r="C51" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E51" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F51" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="C51" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D51" s="5">
-        <v>410</v>
-      </c>
-      <c r="E51" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F51" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="10" t="s">
+      <c r="B52" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="C52" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E52" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F52" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="C52" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D52" s="5">
-        <v>410</v>
-      </c>
-      <c r="E52" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F52" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="10" t="s">
+      <c r="B53" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="C53" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E53" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F53" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="C53" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D53" s="5">
-        <v>410</v>
-      </c>
-      <c r="E53" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F53" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="10" t="s">
+      <c r="B54" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="C54" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E54" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F54" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C54" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D54" s="5">
-        <v>410</v>
-      </c>
-      <c r="E54" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F54" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="10" t="s">
+      <c r="B55" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B55" s="10" t="s">
+      <c r="C55" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E55" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F55" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C55" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D55" s="5">
-        <v>410</v>
-      </c>
-      <c r="E55" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F55" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10" t="s">
+      <c r="B56" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B56" s="10" t="s">
+      <c r="C56" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E56" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F56" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C56" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D56" s="5">
-        <v>410</v>
-      </c>
-      <c r="E56" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F56" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="10" t="s">
+      <c r="B57" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="10" t="s">
+      <c r="C57" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F57" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C57" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D57" s="5">
-        <v>410</v>
-      </c>
-      <c r="E57" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F57" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="10" t="s">
+      <c r="B58" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B58" s="10" t="s">
+      <c r="C58" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F58" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="C58" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D58" s="5">
-        <v>410</v>
-      </c>
-      <c r="E58" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="10" t="s">
+      <c r="B59" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F59" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B59" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="C59" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D59" s="5">
-        <v>410</v>
-      </c>
-      <c r="E59" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F59" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="10" t="s">
+      <c r="B60" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B60" s="10" t="s">
+      <c r="C60" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="C60" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D60" s="5">
-        <v>410</v>
-      </c>
-      <c r="E60" s="5">
-        <v>410999</v>
-      </c>
-      <c r="F60" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="10" t="s">
+      <c r="B61" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B61" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C61" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D61" s="5">
-        <v>410</v>
-      </c>
-      <c r="E61" s="5">
-        <v>410999</v>
+      <c r="C61" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>134</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2050,170 +2045,170 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>123</v>
-      </c>
       <c r="F1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>67</v>
-      </c>
       <c r="C2" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="C3" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>71</v>
-      </c>
       <c r="C4" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>73</v>
-      </c>
       <c r="C5" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="C6" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>77</v>
-      </c>
       <c r="C7" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="C8" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>89</v>
-      </c>
       <c r="C9" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>91</v>
-      </c>
       <c r="C10" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>93</v>
-      </c>
       <c r="C11" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="C12" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2244,27 +2239,27 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>123</v>
-      </c>
       <c r="F1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>87</v>
-      </c>
       <c r="C2" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D2" s="5">
         <v>410</v>
@@ -2273,18 +2268,18 @@
         <v>410999</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>95</v>
-      </c>
       <c r="C3" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D3" s="5">
         <v>410</v>
@@ -2293,18 +2288,18 @@
         <v>410999</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="C4" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D4" s="5">
         <v>410</v>
@@ -2313,18 +2308,18 @@
         <v>410999</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>101</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D5" s="5">
         <v>410</v>
@@ -2333,18 +2328,18 @@
         <v>410999</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>103</v>
-      </c>
       <c r="C6" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D6" s="5">
         <v>410</v>
@@ -2353,18 +2348,18 @@
         <v>410999</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>105</v>
-      </c>
       <c r="C7" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D7" s="5">
         <v>410</v>
@@ -2373,18 +2368,18 @@
         <v>410999</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>107</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D8" s="5">
         <v>410</v>
@@ -2393,18 +2388,18 @@
         <v>410999</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>109</v>
-      </c>
       <c r="C9" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D9" s="5">
         <v>410</v>
@@ -2413,18 +2408,18 @@
         <v>410999</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>111</v>
-      </c>
       <c r="C10" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D10" s="5">
         <v>410</v>
@@ -2433,18 +2428,18 @@
         <v>410999</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>113</v>
-      </c>
       <c r="C11" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D11" s="5">
         <v>410</v>
@@ -2453,18 +2448,18 @@
         <v>410999</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>115</v>
-      </c>
       <c r="C12" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D12" s="5">
         <v>410</v>
@@ -2473,18 +2468,18 @@
         <v>410999</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D13" s="5">
         <v>410</v>
@@ -2493,18 +2488,18 @@
         <v>410999</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="14" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>118</v>
-      </c>
       <c r="C14" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D14" s="5">
         <v>410</v>
@@ -2513,18 +2508,18 @@
         <v>410999</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>120</v>
-      </c>
       <c r="C15" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D15" s="5">
         <v>410</v>
@@ -2533,7 +2528,7 @@
         <v>410999</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>